<commit_message>
Reporting for wealth simulation charts + start adding He Kelly and Manela Capital Ratio Factor
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/python/epsilonPhi/core/dataModel/dataSources/futures/futures_info/CL_.xlsx
+++ b/epsilon-phi-core/src/python/epsilonPhi/core/dataModel/dataSources/futures/futures_info/CL_.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/repo/epsilon-psi/epsilon-phi-core/src/python/epsilonPhi/core/dataModel/dataSources/futures/futures_info/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/python/epsilonPhi/core/dataModel/dataSources/futures/futures_info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5717B5-9172-B543-AEC5-0BB7992DBDB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{549FE1FA-6155-BF4E-8400-779469A1FB6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34560" yWindow="1720" windowWidth="28080" windowHeight="20540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -10180,6 +10180,10 @@
   <dimension ref="A1:AE634"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="2" max="2" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="20" max="20" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="17.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>